<commit_message>
Vendor forms, ERP backlog, and deck update
Use the ERP history for past and future:
- vendor_forms.py: per-PO acknowledgment form (locked PO lines, required
  response per line, real delivery date, reason codes) and a per-vendor
  supplier information pack pre-filled from 8 months of ERP history
- Returned forms load into the daily check: declined lines and incomplete
  lines get their own issue types instead of 'possible dropped line';
  vendor-declared part numbers go to the review queue
- Supplier pack returns: validation, reply email, lead-time gap report,
  stored in a new vendor_profiles table
- Old Open Balances from the ERP (28k past-due open qty) in the
  workbook and on the Chase page
- Desk app 'Vendor forms' page; 14 new tests (58 total)
- Deck: new 'fix it at the source' slide; README section 4; submission zip

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6V2KMLCSVtUq6RnfYMNep
</commit_message>
<xml_diff>
--- a/Beacon Superday-Submission/output/PO_Confirmation_Check_2026-05-17.xlsx
+++ b/Beacon Superday-Submission/output/PO_Confirmation_Check_2026-05-17.xlsx
@@ -14,12 +14,14 @@
     <sheet name="Draft Emails" sheetId="5" r:id="rId5"/>
     <sheet name="Documents" sheetId="6" r:id="rId6"/>
     <sheet name="PN Crosswalk" sheetId="7" r:id="rId7"/>
-    <sheet name="Run Summary" sheetId="8" r:id="rId8"/>
+    <sheet name="Old Open Balances" sheetId="8" r:id="rId8"/>
+    <sheet name="Run Summary" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Action List'!$A$4:$AA$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All PO Lines'!$A$1:$AA$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Documents!$A$1:$K$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Old Open Balances'!$A$3:$M$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review Required'!$A$3:$M$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1458" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1675" uniqueCount="488">
   <si>
     <t>PO confirmation check - as of 05/17/2026:  44 open PO lines | 23 items need attention | 22 lines fully clean</t>
   </si>
@@ -629,6 +631,27 @@
     <t>Vendor PN 'OST-CAR-A-100' is not in the approved crosswalk. It matched PO line 2 on qty+price+line no. ERP history knows this part from this vendor as WZ-HM-EIN - vendor may have renumbered.</t>
   </si>
   <si>
+    <t>OCR spot-check</t>
+  </si>
+  <si>
+    <t>PO-4500050023</t>
+  </si>
+  <si>
+    <t>Precipitation heat treat A286, per lb qty 750.0 promise 05/23/2026</t>
+  </si>
+  <si>
+    <t>Tesseract OCR</t>
+  </si>
+  <si>
+    <t>Scanned document; numbers were read by OCR.</t>
+  </si>
+  <si>
+    <t>Glance at the PDF and confirm qty/date match what's shown here.</t>
+  </si>
+  <si>
+    <t>continental_04.pdf</t>
+  </si>
+  <si>
     <t>Date interpretation</t>
   </si>
   <si>
@@ -645,27 +668,6 @@
   </si>
   <si>
     <t>Ask vendor for a specific ship date.</t>
-  </si>
-  <si>
-    <t>OCR spot-check</t>
-  </si>
-  <si>
-    <t>PO-4500050023</t>
-  </si>
-  <si>
-    <t>Precipitation heat treat A286, per lb qty 750.0 promise 05/23/2026</t>
-  </si>
-  <si>
-    <t>Tesseract OCR</t>
-  </si>
-  <si>
-    <t>Scanned document; numbers were read by OCR.</t>
-  </si>
-  <si>
-    <t>Glance at the PDF and confirm qty/date match what's shown here.</t>
-  </si>
-  <si>
-    <t>continental_04.pdf</t>
   </si>
   <si>
     <t>Solution treat + age, per lb qty 350.0 promise 05/09/2026</t>
@@ -1316,6 +1318,159 @@
     <t>2026-03-24</t>
   </si>
   <si>
+    <t>From the ERP: PO lines past their required date with quantity still open (40 lines, $127,965). Months-old short-shipped balances are usually vendor short-ships nobody closed - chase the balance or short-close the line so MRP stops counting on it.</t>
+  </si>
+  <si>
+    <t>Part</t>
+  </si>
+  <si>
+    <t>Ordered</t>
+  </si>
+  <si>
+    <t>Received</t>
+  </si>
+  <si>
+    <t>Open balance</t>
+  </si>
+  <si>
+    <t>Balance $</t>
+  </si>
+  <si>
+    <t>Days past due</t>
+  </si>
+  <si>
+    <t>What it is</t>
+  </si>
+  <si>
+    <t>Last receipt</t>
+  </si>
+  <si>
+    <t>Suggested action</t>
+  </si>
+  <si>
+    <t>Nothing received</t>
+  </si>
+  <si>
+    <t>Chase: nothing received yet.</t>
+  </si>
+  <si>
+    <t>PO-4500045503</t>
+  </si>
+  <si>
+    <t>Short-shipped balance left open</t>
+  </si>
+  <si>
+    <t>Probably never shipping: confirm with vendor and short-close.</t>
+  </si>
+  <si>
+    <t>PO-4500045921</t>
+  </si>
+  <si>
+    <t>PO-4500046944</t>
+  </si>
+  <si>
+    <t>HT-STRESS</t>
+  </si>
+  <si>
+    <t>PO-4500045662</t>
+  </si>
+  <si>
+    <t>Ask vendor if the balance will ship; if not, short-close the line.</t>
+  </si>
+  <si>
+    <t>PO-4500045901</t>
+  </si>
+  <si>
+    <t>PO-4500045536</t>
+  </si>
+  <si>
+    <t>PO-4500045694</t>
+  </si>
+  <si>
+    <t>PO-4500045902</t>
+  </si>
+  <si>
+    <t>PO-4500046876</t>
+  </si>
+  <si>
+    <t>PO-4500046185</t>
+  </si>
+  <si>
+    <t>PO-4500046863</t>
+  </si>
+  <si>
+    <t>BAR-4130-312</t>
+  </si>
+  <si>
+    <t>PO-4500046202</t>
+  </si>
+  <si>
+    <t>PO-4500046523</t>
+  </si>
+  <si>
+    <t>PO-4500046323</t>
+  </si>
+  <si>
+    <t>PO-4500045999</t>
+  </si>
+  <si>
+    <t>PO-4500046357</t>
+  </si>
+  <si>
+    <t>PO-4500046120</t>
+  </si>
+  <si>
+    <t>PO-4500046226</t>
+  </si>
+  <si>
+    <t>PO-4500046787</t>
+  </si>
+  <si>
+    <t>PO-4500046799</t>
+  </si>
+  <si>
+    <t>PO-4500046166</t>
+  </si>
+  <si>
+    <t>PO-4500046419</t>
+  </si>
+  <si>
+    <t>PO-4500046755</t>
+  </si>
+  <si>
+    <t>PLAT-ZN</t>
+  </si>
+  <si>
+    <t>PO-4500046083</t>
+  </si>
+  <si>
+    <t>PO-4500046704</t>
+  </si>
+  <si>
+    <t>PO-4500046429</t>
+  </si>
+  <si>
+    <t>PO-4500046363</t>
+  </si>
+  <si>
+    <t>PO-4500046515</t>
+  </si>
+  <si>
+    <t>PO-4500047234</t>
+  </si>
+  <si>
+    <t>PO-4500046586</t>
+  </si>
+  <si>
+    <t>PO-4500046481</t>
+  </si>
+  <si>
+    <t>PO-4500047308</t>
+  </si>
+  <si>
+    <t>PO-4500047214</t>
+  </si>
+  <si>
     <t>Run summary and validation checks - as of 05/17/2026</t>
   </si>
   <si>
@@ -1328,6 +1483,9 @@
     <t xml:space="preserve">  read by OCR (scans)</t>
   </si>
   <si>
+    <t xml:space="preserve">  Beacon forms (no reading needed)</t>
+  </si>
+  <si>
     <t xml:space="preserve">  unreadable (manual)</t>
   </si>
   <si>
@@ -1350,6 +1508,12 @@
   </si>
   <si>
     <t xml:space="preserve">  acknowledged without qty/date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  declined by vendor (Beacon form)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  incomplete on Beacon form</t>
   </si>
   <si>
     <t>Priority 1 (act today) lines</t>
@@ -3820,20 +3984,14 @@
         <v>200</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>66</v>
+        <v>94</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D9" s="2">
-        <v>1</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F9" s="2" t="s">
         <v>201</v>
       </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
         <v>202</v>
       </c>
@@ -3850,12 +4008,12 @@
         <v>205</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>72</v>
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="2" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>66</v>
@@ -3864,28 +4022,28 @@
         <v>67</v>
       </c>
       <c r="D10" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>81</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>72</v>
@@ -3893,39 +4051,45 @@
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>94</v>
+        <v>66</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
+        <v>67</v>
+      </c>
+      <c r="D11" s="2">
+        <v>2</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>208</v>
+      </c>
       <c r="G11" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>81</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>212</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="2" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>94</v>
@@ -3940,16 +4104,16 @@
         <v>213</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>81</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>131</v>
@@ -3957,7 +4121,7 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="2" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>94</v>
@@ -3972,16 +4136,16 @@
         <v>214</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>81</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>127</v>
@@ -3989,7 +4153,7 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="2" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>94</v>
@@ -4004,16 +4168,16 @@
         <v>215</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>81</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>99</v>
@@ -6426,7 +6590,7 @@
         <v>94</v>
       </c>
       <c r="C33" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="D33">
         <v>1</v>
@@ -6474,7 +6638,7 @@
         <v>54</v>
       </c>
       <c r="Y33" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="Z33" s="8">
         <v>46165</v>
@@ -8203,7 +8367,7 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="B14" t="s">
         <v>94</v>
@@ -8218,7 +8382,7 @@
         <v>310</v>
       </c>
       <c r="F14" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="G14" s="8">
         <v>46154</v>
@@ -9374,7 +9538,1693 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:M43"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="6.7109375" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" customWidth="1"/>
+    <col min="5" max="6" width="10.7109375" customWidth="1"/>
+    <col min="7" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" customWidth="1"/>
+    <col min="11" max="11" width="30.7109375" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="13" width="50.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="45" customHeight="1">
+      <c r="A1" s="2" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E4" s="5">
+        <v>25</v>
+      </c>
+      <c r="F4" s="5">
+        <v>0</v>
+      </c>
+      <c r="G4" s="5">
+        <v>25</v>
+      </c>
+      <c r="H4" s="7">
+        <v>31000</v>
+      </c>
+      <c r="I4" s="8">
+        <v>46157</v>
+      </c>
+      <c r="J4" s="5">
+        <v>2</v>
+      </c>
+      <c r="K4" t="s">
+        <v>423</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>425</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>243</v>
+      </c>
+      <c r="E5" s="5">
+        <v>22400</v>
+      </c>
+      <c r="F5" s="5">
+        <v>21207</v>
+      </c>
+      <c r="G5" s="5">
+        <v>1193</v>
+      </c>
+      <c r="H5" s="7">
+        <v>26842.5</v>
+      </c>
+      <c r="I5" s="8">
+        <v>45944</v>
+      </c>
+      <c r="J5" s="5">
+        <v>215</v>
+      </c>
+      <c r="K5" t="s">
+        <v>426</v>
+      </c>
+      <c r="L5" s="8">
+        <v>45938</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>428</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>243</v>
+      </c>
+      <c r="E6" s="5">
+        <v>6700</v>
+      </c>
+      <c r="F6" s="5">
+        <v>6147</v>
+      </c>
+      <c r="G6" s="5">
+        <v>553</v>
+      </c>
+      <c r="H6" s="7">
+        <v>12442.5</v>
+      </c>
+      <c r="I6" s="8">
+        <v>46017</v>
+      </c>
+      <c r="J6" s="5">
+        <v>142</v>
+      </c>
+      <c r="K6" t="s">
+        <v>426</v>
+      </c>
+      <c r="L6" s="8">
+        <v>46017</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" t="s">
+        <v>429</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>430</v>
+      </c>
+      <c r="E7" s="5">
+        <v>5800</v>
+      </c>
+      <c r="F7" s="5">
+        <v>0</v>
+      </c>
+      <c r="G7" s="5">
+        <v>5800</v>
+      </c>
+      <c r="H7" s="7">
+        <v>9280</v>
+      </c>
+      <c r="I7" s="8">
+        <v>46157</v>
+      </c>
+      <c r="J7" s="5">
+        <v>2</v>
+      </c>
+      <c r="K7" t="s">
+        <v>423</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" t="s">
+        <v>431</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>228</v>
+      </c>
+      <c r="E8" s="5">
+        <v>21600</v>
+      </c>
+      <c r="F8" s="5">
+        <v>20419</v>
+      </c>
+      <c r="G8" s="5">
+        <v>1181</v>
+      </c>
+      <c r="H8" s="7">
+        <v>9259.039999999999</v>
+      </c>
+      <c r="I8" s="8">
+        <v>46118</v>
+      </c>
+      <c r="J8" s="5">
+        <v>41</v>
+      </c>
+      <c r="K8" t="s">
+        <v>426</v>
+      </c>
+      <c r="L8" s="8">
+        <v>46113</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>433</v>
+      </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>228</v>
+      </c>
+      <c r="E9" s="5">
+        <v>11800</v>
+      </c>
+      <c r="F9" s="5">
+        <v>10723</v>
+      </c>
+      <c r="G9" s="5">
+        <v>1077</v>
+      </c>
+      <c r="H9" s="7">
+        <v>8443.68</v>
+      </c>
+      <c r="I9" s="8">
+        <v>46084</v>
+      </c>
+      <c r="J9" s="5">
+        <v>75</v>
+      </c>
+      <c r="K9" t="s">
+        <v>426</v>
+      </c>
+      <c r="L9" s="8">
+        <v>46084</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" t="s">
+        <v>434</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="5">
+        <v>20100</v>
+      </c>
+      <c r="F10" s="5">
+        <v>18094</v>
+      </c>
+      <c r="G10" s="5">
+        <v>2006</v>
+      </c>
+      <c r="H10" s="7">
+        <v>7863.52</v>
+      </c>
+      <c r="I10" s="8">
+        <v>46136</v>
+      </c>
+      <c r="J10" s="5">
+        <v>23</v>
+      </c>
+      <c r="K10" t="s">
+        <v>426</v>
+      </c>
+      <c r="L10" s="8">
+        <v>46133</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
+      <c r="A11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" t="s">
+        <v>435</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>228</v>
+      </c>
+      <c r="E11" s="5">
+        <v>8500</v>
+      </c>
+      <c r="F11" s="5">
+        <v>7788</v>
+      </c>
+      <c r="G11" s="5">
+        <v>712</v>
+      </c>
+      <c r="H11" s="7">
+        <v>5582.08</v>
+      </c>
+      <c r="I11" s="8">
+        <v>46107</v>
+      </c>
+      <c r="J11" s="5">
+        <v>52</v>
+      </c>
+      <c r="K11" t="s">
+        <v>426</v>
+      </c>
+      <c r="L11" s="8">
+        <v>46100</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
+      <c r="A12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" t="s">
+        <v>436</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12" t="s">
+        <v>243</v>
+      </c>
+      <c r="E12" s="5">
+        <v>3200</v>
+      </c>
+      <c r="F12" s="5">
+        <v>2963</v>
+      </c>
+      <c r="G12" s="5">
+        <v>237</v>
+      </c>
+      <c r="H12" s="7">
+        <v>5332.5</v>
+      </c>
+      <c r="I12" s="8">
+        <v>46093</v>
+      </c>
+      <c r="J12" s="5">
+        <v>66</v>
+      </c>
+      <c r="K12" t="s">
+        <v>426</v>
+      </c>
+      <c r="L12" s="8">
+        <v>46093</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="A13" t="s">
+        <v>94</v>
+      </c>
+      <c r="B13" t="s">
+        <v>437</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13" t="s">
+        <v>123</v>
+      </c>
+      <c r="E13" s="5">
+        <v>8350</v>
+      </c>
+      <c r="F13" s="5">
+        <v>7960</v>
+      </c>
+      <c r="G13" s="5">
+        <v>390</v>
+      </c>
+      <c r="H13" s="7">
+        <v>1209</v>
+      </c>
+      <c r="I13" s="8">
+        <v>46008</v>
+      </c>
+      <c r="J13" s="5">
+        <v>151</v>
+      </c>
+      <c r="K13" t="s">
+        <v>426</v>
+      </c>
+      <c r="L13" s="8">
+        <v>46025</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
+      <c r="A14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B14" t="s">
+        <v>438</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14" t="s">
+        <v>396</v>
+      </c>
+      <c r="E14" s="5">
+        <v>21900</v>
+      </c>
+      <c r="F14" s="5">
+        <v>19888</v>
+      </c>
+      <c r="G14" s="5">
+        <v>2012</v>
+      </c>
+      <c r="H14" s="7">
+        <v>1106.6</v>
+      </c>
+      <c r="I14" s="8">
+        <v>46001</v>
+      </c>
+      <c r="J14" s="5">
+        <v>158</v>
+      </c>
+      <c r="K14" t="s">
+        <v>426</v>
+      </c>
+      <c r="L14" s="8">
+        <v>46001</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
+      <c r="A15" t="s">
+        <v>94</v>
+      </c>
+      <c r="B15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" t="s">
+        <v>123</v>
+      </c>
+      <c r="E15" s="5">
+        <v>350</v>
+      </c>
+      <c r="F15" s="5">
+        <v>0</v>
+      </c>
+      <c r="G15" s="5">
+        <v>350</v>
+      </c>
+      <c r="H15" s="7">
+        <v>1085</v>
+      </c>
+      <c r="I15" s="8">
+        <v>46151</v>
+      </c>
+      <c r="J15" s="5">
+        <v>8</v>
+      </c>
+      <c r="K15" t="s">
+        <v>423</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
+      <c r="A16" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" t="s">
+        <v>122</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>123</v>
+      </c>
+      <c r="E16" s="5">
+        <v>350</v>
+      </c>
+      <c r="F16" s="5">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5">
+        <v>350</v>
+      </c>
+      <c r="H16" s="7">
+        <v>1085</v>
+      </c>
+      <c r="I16" s="8">
+        <v>46149</v>
+      </c>
+      <c r="J16" s="5">
+        <v>10</v>
+      </c>
+      <c r="K16" t="s">
+        <v>423</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
+      <c r="A17" t="s">
+        <v>94</v>
+      </c>
+      <c r="B17" t="s">
+        <v>439</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>123</v>
+      </c>
+      <c r="E17" s="5">
+        <v>6900</v>
+      </c>
+      <c r="F17" s="5">
+        <v>6566</v>
+      </c>
+      <c r="G17" s="5">
+        <v>334</v>
+      </c>
+      <c r="H17" s="7">
+        <v>1035.4</v>
+      </c>
+      <c r="I17" s="8">
+        <v>46155</v>
+      </c>
+      <c r="J17" s="5">
+        <v>4</v>
+      </c>
+      <c r="K17" t="s">
+        <v>426</v>
+      </c>
+      <c r="L17" s="8">
+        <v>46159</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
+      <c r="A18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" t="s">
+        <v>433</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="s">
+        <v>440</v>
+      </c>
+      <c r="E18" s="5">
+        <v>5300</v>
+      </c>
+      <c r="F18" s="5">
+        <v>4970</v>
+      </c>
+      <c r="G18" s="5">
+        <v>330</v>
+      </c>
+      <c r="H18" s="7">
+        <v>940.5</v>
+      </c>
+      <c r="I18" s="8">
+        <v>46084</v>
+      </c>
+      <c r="J18" s="5">
+        <v>75</v>
+      </c>
+      <c r="K18" t="s">
+        <v>426</v>
+      </c>
+      <c r="L18" s="8">
+        <v>46085</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
+      <c r="A19" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19">
+        <v>2</v>
+      </c>
+      <c r="D19" t="s">
+        <v>76</v>
+      </c>
+      <c r="E19" s="5">
+        <v>50</v>
+      </c>
+      <c r="F19" s="5">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5">
+        <v>50</v>
+      </c>
+      <c r="H19" s="7">
+        <v>910</v>
+      </c>
+      <c r="I19" s="8">
+        <v>46157</v>
+      </c>
+      <c r="J19" s="5">
+        <v>2</v>
+      </c>
+      <c r="K19" t="s">
+        <v>423</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
+      <c r="A20" t="s">
+        <v>110</v>
+      </c>
+      <c r="B20" t="s">
+        <v>441</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20" t="s">
+        <v>150</v>
+      </c>
+      <c r="E20" s="5">
+        <v>18200</v>
+      </c>
+      <c r="F20" s="5">
+        <v>17279</v>
+      </c>
+      <c r="G20" s="5">
+        <v>921</v>
+      </c>
+      <c r="H20" s="7">
+        <v>773.64</v>
+      </c>
+      <c r="I20" s="8">
+        <v>46072</v>
+      </c>
+      <c r="J20" s="5">
+        <v>87</v>
+      </c>
+      <c r="K20" t="s">
+        <v>426</v>
+      </c>
+      <c r="L20" s="8">
+        <v>46076</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
+      <c r="A21" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" t="s">
+        <v>442</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21" t="s">
+        <v>86</v>
+      </c>
+      <c r="E21" s="5">
+        <v>8350</v>
+      </c>
+      <c r="F21" s="5">
+        <v>0</v>
+      </c>
+      <c r="G21" s="5">
+        <v>8350</v>
+      </c>
+      <c r="H21" s="7">
+        <v>668</v>
+      </c>
+      <c r="I21" s="8">
+        <v>46157</v>
+      </c>
+      <c r="J21" s="5">
+        <v>2</v>
+      </c>
+      <c r="K21" t="s">
+        <v>423</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
+      <c r="A22" t="s">
+        <v>110</v>
+      </c>
+      <c r="B22" t="s">
+        <v>443</v>
+      </c>
+      <c r="C22">
+        <v>2</v>
+      </c>
+      <c r="D22" t="s">
+        <v>150</v>
+      </c>
+      <c r="E22" s="5">
+        <v>9500</v>
+      </c>
+      <c r="F22" s="5">
+        <v>8793</v>
+      </c>
+      <c r="G22" s="5">
+        <v>707</v>
+      </c>
+      <c r="H22" s="7">
+        <v>593.88</v>
+      </c>
+      <c r="I22" s="8">
+        <v>46056</v>
+      </c>
+      <c r="J22" s="5">
+        <v>103</v>
+      </c>
+      <c r="K22" t="s">
+        <v>426</v>
+      </c>
+      <c r="L22" s="8">
+        <v>46063</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13">
+      <c r="A23" t="s">
+        <v>110</v>
+      </c>
+      <c r="B23" t="s">
+        <v>444</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23" t="s">
+        <v>150</v>
+      </c>
+      <c r="E23" s="5">
+        <v>16900</v>
+      </c>
+      <c r="F23" s="5">
+        <v>16247</v>
+      </c>
+      <c r="G23" s="5">
+        <v>653</v>
+      </c>
+      <c r="H23" s="7">
+        <v>548.52</v>
+      </c>
+      <c r="I23" s="8">
+        <v>45961</v>
+      </c>
+      <c r="J23" s="5">
+        <v>198</v>
+      </c>
+      <c r="K23" t="s">
+        <v>426</v>
+      </c>
+      <c r="L23" s="8">
+        <v>45955</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
+      <c r="A24" t="s">
+        <v>110</v>
+      </c>
+      <c r="B24" t="s">
+        <v>445</v>
+      </c>
+      <c r="C24">
+        <v>2</v>
+      </c>
+      <c r="D24" t="s">
+        <v>396</v>
+      </c>
+      <c r="E24" s="5">
+        <v>8800</v>
+      </c>
+      <c r="F24" s="5">
+        <v>8055</v>
+      </c>
+      <c r="G24" s="5">
+        <v>745</v>
+      </c>
+      <c r="H24" s="7">
+        <v>409.7500000000001</v>
+      </c>
+      <c r="I24" s="8">
+        <v>46042</v>
+      </c>
+      <c r="J24" s="5">
+        <v>117</v>
+      </c>
+      <c r="K24" t="s">
+        <v>426</v>
+      </c>
+      <c r="L24" s="8">
+        <v>46032</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13">
+      <c r="A25" t="s">
+        <v>110</v>
+      </c>
+      <c r="B25" t="s">
+        <v>446</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25" t="s">
+        <v>396</v>
+      </c>
+      <c r="E25" s="5">
+        <v>14900</v>
+      </c>
+      <c r="F25" s="5">
+        <v>14390</v>
+      </c>
+      <c r="G25" s="5">
+        <v>510</v>
+      </c>
+      <c r="H25" s="7">
+        <v>280.5</v>
+      </c>
+      <c r="I25" s="8">
+        <v>46140</v>
+      </c>
+      <c r="J25" s="5">
+        <v>19</v>
+      </c>
+      <c r="K25" t="s">
+        <v>426</v>
+      </c>
+      <c r="L25" s="8">
+        <v>46136</v>
+      </c>
+      <c r="M25" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13">
+      <c r="A26" t="s">
+        <v>110</v>
+      </c>
+      <c r="B26" t="s">
+        <v>447</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26" t="s">
+        <v>155</v>
+      </c>
+      <c r="E26" s="5">
+        <v>14100</v>
+      </c>
+      <c r="F26" s="5">
+        <v>13534</v>
+      </c>
+      <c r="G26" s="5">
+        <v>566</v>
+      </c>
+      <c r="H26" s="7">
+        <v>232.06</v>
+      </c>
+      <c r="I26" s="8">
+        <v>45967</v>
+      </c>
+      <c r="J26" s="5">
+        <v>192</v>
+      </c>
+      <c r="K26" t="s">
+        <v>426</v>
+      </c>
+      <c r="L26" s="8">
+        <v>45969</v>
+      </c>
+      <c r="M26" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
+      <c r="A27" t="s">
+        <v>94</v>
+      </c>
+      <c r="B27" t="s">
+        <v>448</v>
+      </c>
+      <c r="C27">
+        <v>2</v>
+      </c>
+      <c r="D27" t="s">
+        <v>96</v>
+      </c>
+      <c r="E27" s="5">
+        <v>2150</v>
+      </c>
+      <c r="F27" s="5">
+        <v>2056</v>
+      </c>
+      <c r="G27" s="5">
+        <v>94</v>
+      </c>
+      <c r="H27" s="7">
+        <v>225.6</v>
+      </c>
+      <c r="I27" s="8">
+        <v>45954</v>
+      </c>
+      <c r="J27" s="5">
+        <v>205</v>
+      </c>
+      <c r="K27" t="s">
+        <v>426</v>
+      </c>
+      <c r="L27" s="8">
+        <v>45953</v>
+      </c>
+      <c r="M27" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13">
+      <c r="A28" t="s">
+        <v>84</v>
+      </c>
+      <c r="B28" t="s">
+        <v>270</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28" t="s">
+        <v>86</v>
+      </c>
+      <c r="E28" s="5">
+        <v>2500</v>
+      </c>
+      <c r="F28" s="5">
+        <v>0</v>
+      </c>
+      <c r="G28" s="5">
+        <v>2500</v>
+      </c>
+      <c r="H28" s="7">
+        <v>200</v>
+      </c>
+      <c r="I28" s="8">
+        <v>46155</v>
+      </c>
+      <c r="J28" s="5">
+        <v>4</v>
+      </c>
+      <c r="K28" t="s">
+        <v>423</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
+      <c r="A29" t="s">
+        <v>94</v>
+      </c>
+      <c r="B29" t="s">
+        <v>449</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="D29" t="s">
+        <v>96</v>
+      </c>
+      <c r="E29" s="5">
+        <v>1250</v>
+      </c>
+      <c r="F29" s="5">
+        <v>1201</v>
+      </c>
+      <c r="G29" s="5">
+        <v>49</v>
+      </c>
+      <c r="H29" s="7">
+        <v>117.6</v>
+      </c>
+      <c r="I29" s="8">
+        <v>46015</v>
+      </c>
+      <c r="J29" s="5">
+        <v>144</v>
+      </c>
+      <c r="K29" t="s">
+        <v>426</v>
+      </c>
+      <c r="L29" s="8">
+        <v>46011</v>
+      </c>
+      <c r="M29" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
+      <c r="A30" t="s">
+        <v>110</v>
+      </c>
+      <c r="B30" t="s">
+        <v>450</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="D30" t="s">
+        <v>396</v>
+      </c>
+      <c r="E30" s="5">
+        <v>2400</v>
+      </c>
+      <c r="F30" s="5">
+        <v>2222</v>
+      </c>
+      <c r="G30" s="5">
+        <v>178</v>
+      </c>
+      <c r="H30" s="7">
+        <v>97.90000000000001</v>
+      </c>
+      <c r="I30" s="8">
+        <v>46128</v>
+      </c>
+      <c r="J30" s="5">
+        <v>31</v>
+      </c>
+      <c r="K30" t="s">
+        <v>426</v>
+      </c>
+      <c r="L30" s="8">
+        <v>46124</v>
+      </c>
+      <c r="M30" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
+      <c r="A31" t="s">
+        <v>84</v>
+      </c>
+      <c r="B31" t="s">
+        <v>451</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+      <c r="D31" t="s">
+        <v>261</v>
+      </c>
+      <c r="E31" s="5">
+        <v>7950</v>
+      </c>
+      <c r="F31" s="5">
+        <v>7186</v>
+      </c>
+      <c r="G31" s="5">
+        <v>764</v>
+      </c>
+      <c r="H31" s="7">
+        <v>84.04000000000001</v>
+      </c>
+      <c r="I31" s="8">
+        <v>46099</v>
+      </c>
+      <c r="J31" s="5">
+        <v>60</v>
+      </c>
+      <c r="K31" t="s">
+        <v>426</v>
+      </c>
+      <c r="L31" s="8">
+        <v>46095</v>
+      </c>
+      <c r="M31" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13">
+      <c r="A32" t="s">
+        <v>84</v>
+      </c>
+      <c r="B32" t="s">
+        <v>452</v>
+      </c>
+      <c r="C32">
+        <v>2</v>
+      </c>
+      <c r="D32" t="s">
+        <v>453</v>
+      </c>
+      <c r="E32" s="5">
+        <v>6350</v>
+      </c>
+      <c r="F32" s="5">
+        <v>5897</v>
+      </c>
+      <c r="G32" s="5">
+        <v>453</v>
+      </c>
+      <c r="H32" s="7">
+        <v>63.42000000000001</v>
+      </c>
+      <c r="I32" s="8">
+        <v>46037</v>
+      </c>
+      <c r="J32" s="5">
+        <v>122</v>
+      </c>
+      <c r="K32" t="s">
+        <v>426</v>
+      </c>
+      <c r="L32" s="8">
+        <v>46036</v>
+      </c>
+      <c r="M32" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13">
+      <c r="A33" t="s">
+        <v>110</v>
+      </c>
+      <c r="B33" t="s">
+        <v>454</v>
+      </c>
+      <c r="C33">
+        <v>1</v>
+      </c>
+      <c r="D33" t="s">
+        <v>150</v>
+      </c>
+      <c r="E33" s="5">
+        <v>1100</v>
+      </c>
+      <c r="F33" s="5">
+        <v>1030</v>
+      </c>
+      <c r="G33" s="5">
+        <v>70</v>
+      </c>
+      <c r="H33" s="7">
+        <v>58.8</v>
+      </c>
+      <c r="I33" s="8">
+        <v>45947</v>
+      </c>
+      <c r="J33" s="5">
+        <v>212</v>
+      </c>
+      <c r="K33" t="s">
+        <v>426</v>
+      </c>
+      <c r="L33" s="8">
+        <v>45941</v>
+      </c>
+      <c r="M33" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13">
+      <c r="A34" t="s">
+        <v>84</v>
+      </c>
+      <c r="B34" t="s">
+        <v>455</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34" t="s">
+        <v>453</v>
+      </c>
+      <c r="E34" s="5">
+        <v>6600</v>
+      </c>
+      <c r="F34" s="5">
+        <v>6198</v>
+      </c>
+      <c r="G34" s="5">
+        <v>402</v>
+      </c>
+      <c r="H34" s="7">
+        <v>56.28000000000001</v>
+      </c>
+      <c r="I34" s="8">
+        <v>45967</v>
+      </c>
+      <c r="J34" s="5">
+        <v>192</v>
+      </c>
+      <c r="K34" t="s">
+        <v>426</v>
+      </c>
+      <c r="L34" s="8">
+        <v>45965</v>
+      </c>
+      <c r="M34" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13">
+      <c r="A35" t="s">
+        <v>84</v>
+      </c>
+      <c r="B35" t="s">
+        <v>456</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="D35" t="s">
+        <v>453</v>
+      </c>
+      <c r="E35" s="5">
+        <v>6950</v>
+      </c>
+      <c r="F35" s="5">
+        <v>6595</v>
+      </c>
+      <c r="G35" s="5">
+        <v>355</v>
+      </c>
+      <c r="H35" s="7">
+        <v>49.7</v>
+      </c>
+      <c r="I35" s="8">
+        <v>46142</v>
+      </c>
+      <c r="J35" s="5">
+        <v>17</v>
+      </c>
+      <c r="K35" t="s">
+        <v>426</v>
+      </c>
+      <c r="L35" s="8">
+        <v>46139</v>
+      </c>
+      <c r="M35" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13">
+      <c r="A36" t="s">
+        <v>110</v>
+      </c>
+      <c r="B36" t="s">
+        <v>457</v>
+      </c>
+      <c r="C36">
+        <v>1</v>
+      </c>
+      <c r="D36" t="s">
+        <v>157</v>
+      </c>
+      <c r="E36" s="5">
+        <v>700</v>
+      </c>
+      <c r="F36" s="5">
+        <v>646</v>
+      </c>
+      <c r="G36" s="5">
+        <v>54</v>
+      </c>
+      <c r="H36" s="7">
+        <v>33.48</v>
+      </c>
+      <c r="I36" s="8">
+        <v>46079</v>
+      </c>
+      <c r="J36" s="5">
+        <v>80</v>
+      </c>
+      <c r="K36" t="s">
+        <v>426</v>
+      </c>
+      <c r="L36" s="8">
+        <v>46086</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
+      <c r="A37" t="s">
+        <v>134</v>
+      </c>
+      <c r="B37" t="s">
+        <v>282</v>
+      </c>
+      <c r="C37">
+        <v>1</v>
+      </c>
+      <c r="D37" t="s">
+        <v>136</v>
+      </c>
+      <c r="E37" s="5">
+        <v>500</v>
+      </c>
+      <c r="F37" s="5">
+        <v>0</v>
+      </c>
+      <c r="G37" s="5">
+        <v>500</v>
+      </c>
+      <c r="H37" s="7">
+        <v>30</v>
+      </c>
+      <c r="I37" s="8">
+        <v>46157</v>
+      </c>
+      <c r="J37" s="5">
+        <v>2</v>
+      </c>
+      <c r="K37" t="s">
+        <v>423</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13">
+      <c r="A38" t="s">
+        <v>84</v>
+      </c>
+      <c r="B38" t="s">
+        <v>458</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="D38" t="s">
+        <v>86</v>
+      </c>
+      <c r="E38" s="5">
+        <v>1200</v>
+      </c>
+      <c r="F38" s="5">
+        <v>1102</v>
+      </c>
+      <c r="G38" s="5">
+        <v>98</v>
+      </c>
+      <c r="H38" s="7">
+        <v>7.84</v>
+      </c>
+      <c r="I38" s="8">
+        <v>46112</v>
+      </c>
+      <c r="J38" s="5">
+        <v>47</v>
+      </c>
+      <c r="K38" t="s">
+        <v>426</v>
+      </c>
+      <c r="L38" s="8">
+        <v>46105</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13">
+      <c r="A39" t="s">
+        <v>134</v>
+      </c>
+      <c r="B39" t="s">
+        <v>459</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="D39" t="s">
+        <v>136</v>
+      </c>
+      <c r="E39" s="5">
+        <v>1760</v>
+      </c>
+      <c r="F39" s="5">
+        <v>1675</v>
+      </c>
+      <c r="G39" s="5">
+        <v>85</v>
+      </c>
+      <c r="H39" s="7">
+        <v>5.1</v>
+      </c>
+      <c r="I39" s="8">
+        <v>46136</v>
+      </c>
+      <c r="J39" s="5">
+        <v>23</v>
+      </c>
+      <c r="K39" t="s">
+        <v>426</v>
+      </c>
+      <c r="L39" s="8">
+        <v>46135</v>
+      </c>
+      <c r="M39" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13">
+      <c r="A40" t="s">
+        <v>84</v>
+      </c>
+      <c r="B40" t="s">
+        <v>460</v>
+      </c>
+      <c r="C40">
+        <v>2</v>
+      </c>
+      <c r="D40" t="s">
+        <v>86</v>
+      </c>
+      <c r="E40" s="5">
+        <v>900</v>
+      </c>
+      <c r="F40" s="5">
+        <v>850</v>
+      </c>
+      <c r="G40" s="5">
+        <v>50</v>
+      </c>
+      <c r="H40" s="7">
+        <v>4</v>
+      </c>
+      <c r="I40" s="8">
+        <v>46013</v>
+      </c>
+      <c r="J40" s="5">
+        <v>146</v>
+      </c>
+      <c r="K40" t="s">
+        <v>426</v>
+      </c>
+      <c r="L40" s="8">
+        <v>46012</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13">
+      <c r="A41" t="s">
+        <v>84</v>
+      </c>
+      <c r="B41" t="s">
+        <v>461</v>
+      </c>
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41" t="s">
+        <v>86</v>
+      </c>
+      <c r="E41" s="5">
+        <v>550</v>
+      </c>
+      <c r="F41" s="5">
+        <v>516</v>
+      </c>
+      <c r="G41" s="5">
+        <v>34</v>
+      </c>
+      <c r="H41" s="7">
+        <v>2.72</v>
+      </c>
+      <c r="I41" s="8">
+        <v>45971</v>
+      </c>
+      <c r="J41" s="5">
+        <v>188</v>
+      </c>
+      <c r="K41" t="s">
+        <v>426</v>
+      </c>
+      <c r="L41" s="8">
+        <v>45968</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13">
+      <c r="A42" t="s">
+        <v>134</v>
+      </c>
+      <c r="B42" t="s">
+        <v>462</v>
+      </c>
+      <c r="C42">
+        <v>1</v>
+      </c>
+      <c r="D42" t="s">
+        <v>143</v>
+      </c>
+      <c r="E42" s="5">
+        <v>200</v>
+      </c>
+      <c r="F42" s="5">
+        <v>186</v>
+      </c>
+      <c r="G42" s="5">
+        <v>14</v>
+      </c>
+      <c r="H42" s="7">
+        <v>2.52</v>
+      </c>
+      <c r="I42" s="8">
+        <v>46078</v>
+      </c>
+      <c r="J42" s="5">
+        <v>81</v>
+      </c>
+      <c r="K42" t="s">
+        <v>426</v>
+      </c>
+      <c r="L42" s="8">
+        <v>46075</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13">
+      <c r="A43" t="s">
+        <v>134</v>
+      </c>
+      <c r="B43" t="s">
+        <v>463</v>
+      </c>
+      <c r="C43">
+        <v>1</v>
+      </c>
+      <c r="D43" t="s">
+        <v>136</v>
+      </c>
+      <c r="E43" s="5">
+        <v>600</v>
+      </c>
+      <c r="F43" s="5">
+        <v>569</v>
+      </c>
+      <c r="G43" s="5">
+        <v>31</v>
+      </c>
+      <c r="H43" s="7">
+        <v>1.86</v>
+      </c>
+      <c r="I43" s="8">
+        <v>46017</v>
+      </c>
+      <c r="J43" s="5">
+        <v>142</v>
+      </c>
+      <c r="K43" t="s">
+        <v>426</v>
+      </c>
+      <c r="L43" s="8">
+        <v>46016</v>
+      </c>
+      <c r="M43" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:M43"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="55.7109375" customWidth="1"/>
@@ -9384,12 +11234,12 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>413</v>
+        <v>464</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>414</v>
+        <v>465</v>
       </c>
       <c r="B3">
         <v>35</v>
@@ -9397,7 +11247,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>415</v>
+        <v>466</v>
       </c>
       <c r="B4">
         <v>31</v>
@@ -9405,7 +11255,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>416</v>
+        <v>467</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -9413,7 +11263,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>417</v>
+        <v>468</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -9421,7 +11271,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>418</v>
+        <v>469</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -9429,15 +11279,15 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>419</v>
+        <v>470</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>420</v>
+        <v>471</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -9445,47 +11295,47 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>286</v>
+        <v>472</v>
       </c>
       <c r="B10">
-        <v>44</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>421</v>
+        <v>286</v>
       </c>
       <c r="B11">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>422</v>
+        <v>473</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>423</v>
+        <v>474</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>424</v>
+        <v>475</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>425</v>
+        <v>476</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -9493,66 +11343,90 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>426</v>
+        <v>477</v>
       </c>
       <c r="B16">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>427</v>
+        <v>478</v>
       </c>
       <c r="B17">
-        <v>13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>288</v>
+        <v>479</v>
       </c>
       <c r="B18">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>428</v>
+        <v>480</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>429</v>
+        <v>481</v>
       </c>
       <c r="B20">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>430</v>
+        <v>288</v>
       </c>
       <c r="B21">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>482</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>483</v>
+      </c>
+      <c r="B23">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>484</v>
+      </c>
+      <c r="B24">
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
-      <c r="A22" s="14" t="s">
-        <v>431</v>
-      </c>
-      <c r="B22" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="14" t="s">
-        <v>433</v>
-      </c>
-      <c r="B23" t="s">
-        <v>432</v>
+    <row r="25" spans="1:2">
+      <c r="A25" s="14" t="s">
+        <v>485</v>
+      </c>
+      <c r="B25" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="14" t="s">
+        <v>487</v>
+      </c>
+      <c r="B26" t="s">
+        <v>486</v>
       </c>
     </row>
   </sheetData>

</xml_diff>